<commit_message>
updated SAD & s2t
</commit_message>
<xml_diff>
--- a/Docs/Source to target mapping.xlsx
+++ b/Docs/Source to target mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20384"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZinukovD\source\repos\Northwind_BI_Solution\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinyk\source\repos\Northwind_BI_Solution\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1886F2E7-3FF5-4AA5-B8B8-AFB8F731415E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2497363C-E546-46FB-A024-5AA919F212D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="558" activeTab="3" xr2:uid="{4088A55A-653F-450D-AAB8-4D657457B3B6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="558" activeTab="1" xr2:uid="{4088A55A-653F-450D-AAB8-4D657457B3B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="2" r:id="rId1"/>
@@ -1024,27 +1024,6 @@
     <t>NOT LOOKUP HASH TABLE</t>
   </si>
   <si>
-    <t>CHECKSUM ( [CompanyName], [ContactName], [ContactTitle], [City], [Country], [Phone], [Fax] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [Date], [DateType], [HolidayName] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [LastName], [FirstName], [Title], [TitleOfCourtesy], [City], [Country] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [ProductName], [CategoryID] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [CategoryName] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [CustomerID], [EmployeeID], [OrderDate], [RequiredDate], [ShippedDate] )</t>
-  </si>
-  <si>
-    <t>CHECKSUM ( [UnitPrice], [Quantity], [Discount] )</t>
-  </si>
-  <si>
     <t>Lookup OrderID in Order Details &amp; Lookup ProductKey in Dimension.Product</t>
   </si>
   <si>
@@ -1121,6 +1100,27 @@
 			FOR JSON PATH, WITHOUT_ARRAY_WRAPPER
 		)
 (DT_NTEXT)"{\"MDS\":[{\"mdm_masterProduct\":" + (ISNULL(MasterProductAllAttributes) ? (DT_NTEXT)"{}" : MasterProductAllAttributes) + (DT_NTEXT)"}],\"DQS\":[{\"dbo_NW_Products\":" + (ISNULL(DQSProductAllAttributes) ? (DT_NTEXT)"{}" : DQSProductAllAttributes) + (DT_NTEXT)"},{\"dbo_NW_Categories\":" + (ISNULL(DQSCategoryAllAttributes) ? (DT_NTEXT)"{}" : DQSCategoryAllAttributes) + (DT_NTEXT)"}]}"</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [DateType], N'' ), N'#', ISNULL ( [HolidayName], N'' ) ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [CompanyName], N'' ), N'#', ISNULL ( [ContactName], N'' ), N'#', ISNULL ( [ContactTitle], N'' ), N'#', ISNULL ( [City], N'' ), N'#', ISNULL ( [Country], N'' ), N'#', ISNULL ( [Phone], N'' ), N'#', ISNULL ( [Fax], N'' ) ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [LastName], N'' ), N'#', ISNULL ( [FirstName], N'' ), N'#', ISNULL ( [Title], N'' ), N'#', ISNULL ( [TitleOfCourtesy], N'' ), N'#', ISNULL ( [City], N'' ), N'#', ISNULL ( [Country], N'' ) ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [ProductName], N'' ), N'#', ISNULL ( [CategoryID], 0 ) ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', ISNULL ( [CategoryName], N'' ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [CustomerID], CAST ( N'' AS NCHAR(5) ) ), N'#', ISNULL ( [EmployeeID], 0 ), N'#', ISNULL ( [OrderDate], DATEFROMPARTS ( 1995, 12, 31 ) ), N'#', ISNULL ( [RequiredDate], DATEFROMPARTS ( 1995, 12, 31 ) ), N'#', ISNULL ( [ShippedDate], DATEFROMPARTS ( 1995, 12, 31 ) ) ) ) AS VARBINARY(64) )</t>
+  </si>
+  <si>
+    <t>CAST ( HASHBYTES ( N'SHA2_512', CONCAT ( ISNULL ( [UnitPrice], CAST ( 0 AS MONEY ) ), N'#', ISNULL ( [Quantity], CAST ( 0 AS SMALLINT ) ), N'#', ISNULL ( [Discount], CAST ( 0 AS REAL ) ) ) ) AS VARBINARY(64) )</t>
   </si>
 </sst>
 </file>
@@ -1371,13 +1371,24 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1389,22 +1400,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="20% - Accent1" xfId="3" builtinId="30"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="20% — акцент1" xfId="3" builtinId="30"/>
     <cellStyle name="Акцент3 2" xfId="2" xr:uid="{72B9F317-F5C0-45A7-AA7C-0F44C45D1FF6}"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="1" xr:uid="{A125878E-94C1-497A-B7A1-BCB52D1AE9BA}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1421,9 +1421,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1461,7 +1461,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1567,7 +1567,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1709,7 +1709,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1752,47 +1752,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="33" t="s">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="34" t="s">
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="34"/>
-      <c r="R1" s="34"/>
-      <c r="S1" s="34"/>
-      <c r="T1" s="33" t="s">
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="U1" s="33"/>
-      <c r="V1" s="33"/>
-      <c r="W1" s="33"/>
-      <c r="X1" s="33"/>
-      <c r="Y1" s="32" t="s">
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="34"/>
+      <c r="Y1" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="32"/>
+      <c r="Z1" s="36"/>
+      <c r="AA1" s="36"/>
+      <c r="AB1" s="36"/>
+      <c r="AC1" s="36"/>
     </row>
     <row r="2" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -2527,16 +2527,16 @@
         <v>10</v>
       </c>
       <c r="Z12" t="s">
-        <v>341</v>
-      </c>
-      <c r="AA12" s="41" t="s">
+        <v>334</v>
+      </c>
+      <c r="AA12" s="32" t="s">
         <v>61</v>
       </c>
       <c r="AB12" t="s">
         <v>12</v>
       </c>
-      <c r="AC12" s="42" t="s">
-        <v>342</v>
+      <c r="AC12" s="33" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
@@ -2717,7 +2717,7 @@
         <v>325</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
@@ -4652,47 +4652,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="36" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="35" t="s">
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="36" t="s">
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="35" t="s">
+      <c r="P1" s="41"/>
+      <c r="Q1" s="41"/>
+      <c r="R1" s="41"/>
+      <c r="S1" s="41"/>
+      <c r="T1" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="37" t="s">
+      <c r="U1" s="40"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="40"/>
+      <c r="X1" s="40"/>
+      <c r="Y1" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="37"/>
-      <c r="AA1" s="37"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="37"/>
+      <c r="Z1" s="42"/>
+      <c r="AA1" s="42"/>
+      <c r="AB1" s="42"/>
+      <c r="AC1" s="42"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
@@ -6352,7 +6352,7 @@
         <v>325</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="J40" s="26"/>
       <c r="K40" s="26"/>
@@ -7585,47 +7585,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="33" t="s">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="38" t="s">
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="40"/>
-      <c r="T1" s="33" t="s">
+      <c r="P1" s="38"/>
+      <c r="Q1" s="38"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="U1" s="33"/>
-      <c r="V1" s="33"/>
-      <c r="W1" s="33"/>
-      <c r="X1" s="33"/>
-      <c r="Y1" s="32" t="s">
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="34"/>
+      <c r="Y1" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="32"/>
+      <c r="Z1" s="36"/>
+      <c r="AA1" s="36"/>
+      <c r="AB1" s="36"/>
+      <c r="AC1" s="36"/>
     </row>
     <row r="2" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -8194,16 +8194,16 @@
         <v>185</v>
       </c>
       <c r="Z10" t="s">
-        <v>341</v>
-      </c>
-      <c r="AA10" s="41" t="s">
+        <v>334</v>
+      </c>
+      <c r="AA10" s="32" t="s">
         <v>61</v>
       </c>
       <c r="AB10" t="s">
         <v>12</v>
       </c>
-      <c r="AC10" s="42" t="s">
-        <v>343</v>
+      <c r="AC10" s="33" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
@@ -8518,7 +8518,7 @@
         <v>325</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
@@ -10306,47 +10306,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="33" t="s">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="38" t="s">
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="40"/>
-      <c r="T1" s="33" t="s">
+      <c r="P1" s="38"/>
+      <c r="Q1" s="38"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="U1" s="33"/>
-      <c r="V1" s="33"/>
-      <c r="W1" s="33"/>
-      <c r="X1" s="33"/>
-      <c r="Y1" s="32" t="s">
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="34"/>
+      <c r="Y1" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="32"/>
+      <c r="Z1" s="36"/>
+      <c r="AA1" s="36"/>
+      <c r="AB1" s="36"/>
+      <c r="AC1" s="36"/>
     </row>
     <row r="2" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -10691,7 +10691,7 @@
         <v>57</v>
       </c>
       <c r="X6" s="29" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="Y6" s="10" t="s">
         <v>221</v>
@@ -10736,16 +10736,16 @@
         <v>221</v>
       </c>
       <c r="Z7" t="s">
-        <v>341</v>
-      </c>
-      <c r="AA7" s="41" t="s">
+        <v>334</v>
+      </c>
+      <c r="AA7" s="32" t="s">
         <v>61</v>
       </c>
       <c r="AB7" t="s">
         <v>12</v>
       </c>
-      <c r="AC7" s="42" t="s">
-        <v>344</v>
+      <c r="AC7" s="33" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
@@ -10895,7 +10895,7 @@
         <v>325</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
@@ -12291,7 +12291,7 @@
         <v>325</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="J47" s="5"/>
       <c r="K47" s="5"/>
@@ -12801,26 +12801,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="33" t="s">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -12929,7 +12929,7 @@
         <v>301</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -12969,7 +12969,7 @@
         <v>302</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -13009,7 +13009,7 @@
         <v>303</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -13149,7 +13149,7 @@
         <v>300</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -13175,7 +13175,7 @@
         <v>300</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -13201,7 +13201,7 @@
         <v>300</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -13227,7 +13227,7 @@
         <v>300</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -13253,7 +13253,7 @@
         <v>300</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -13358,7 +13358,7 @@
         <v>325</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
@@ -13544,7 +13544,7 @@
         <v>325</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>

</xml_diff>